<commit_message>
chore(backup): weekly snapshot 2026-06-22
</commit_message>
<xml_diff>
--- a/projects/mobile-price-tracker/backups/mobile_plans_2026-06-22.xlsx
+++ b/projects/mobile-price-tracker/backups/mobile_plans_2026-06-22.xlsx
@@ -1554,7 +1554,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -1700,7 +1700,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1910,7 +1910,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -1980,7 +1980,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2190,7 +2190,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -2774,7 +2774,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -2836,7 +2836,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -2898,7 +2898,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -3332,7 +3332,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -3534,7 +3534,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -3884,7 +3884,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -3950,7 +3950,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -4016,7 +4016,7 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -4144,7 +4144,7 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -4206,7 +4206,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -4276,7 +4276,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -4424,7 +4424,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -4498,7 +4498,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -4572,7 +4572,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -4646,7 +4646,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -4716,7 +4716,7 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
@@ -4782,7 +4782,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -4848,7 +4848,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -5120,7 +5120,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -5196,7 +5196,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -5266,7 +5266,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -5336,7 +5336,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -5406,7 +5406,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -5476,7 +5476,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -5546,7 +5546,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -5616,7 +5616,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -5686,7 +5686,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -5756,7 +5756,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -5826,7 +5826,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -5896,7 +5896,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -5966,7 +5966,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -6094,7 +6094,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -6156,7 +6156,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -6218,7 +6218,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -6280,7 +6280,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -6340,7 +6340,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -6402,7 +6402,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -6526,7 +6526,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -6588,7 +6588,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -6712,7 +6712,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -6774,7 +6774,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -6836,7 +6836,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -6898,7 +6898,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -6960,7 +6960,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -7030,7 +7030,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -7170,7 +7170,7 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -7240,7 +7240,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -7310,7 +7310,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -7380,7 +7380,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -7450,7 +7450,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -7516,7 +7516,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -7582,7 +7582,7 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -7648,7 +7648,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -7710,7 +7710,7 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -7772,7 +7772,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -7842,7 +7842,7 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
@@ -7916,7 +7916,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -7990,7 +7990,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -8138,7 +8138,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -8212,7 +8212,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -8282,7 +8282,7 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
@@ -8348,7 +8348,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
@@ -8480,7 +8480,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -8666,7 +8666,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22T18:35:49</t>
+          <t>2026-06-22T22:45:24</t>
         </is>
       </c>
     </row>

</xml_diff>